<commit_message>
UI Refactoring work 09/04/2023 -- UAT observations changes
</commit_message>
<xml_diff>
--- a/ui/src/assets/downloads/uat-scripts.xlsx
+++ b/ui/src/assets/downloads/uat-scripts.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="43">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -30,12 +30,6 @@
   </si>
   <si>
     <t xml:space="preserve">Test Scenario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test Scenario Job ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planned Date</t>
   </si>
   <si>
     <t xml:space="preserve">Step</t>
@@ -247,9 +241,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -359,7 +352,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -381,10 +374,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -417,22 +406,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="4.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="34.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="5.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="6.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="8.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.9"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="14" style="1" width="9.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.9"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1021" min="12" style="1" width="9.18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -469,247 +457,221 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="6" t="n">
-        <v>45183</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="5" t="s">
+      <c r="H2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="E3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="G3" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="5"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="E4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>21</v>
+      </c>
       <c r="G4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="5"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="E5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-    </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="G7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="G8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-    </row>
-    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="G9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="8"/>
-    </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="G10" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
+        <v>15</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -727,19 +689,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="5.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="29.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="25.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="16.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="15.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="29.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="25.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.76"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -776,270 +736,242 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="6" t="n">
-        <v>45220</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>1</v>
+      <c r="F2" s="5" t="s">
+        <v>14</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
       <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="5"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="E3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="G3" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="5"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="E4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="G4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="4" t="n">
+      <c r="C5" s="7"/>
+      <c r="D5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="E5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-    </row>
-    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-    </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="G9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="8"/>
-    </row>
-    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="G11" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
-      <c r="M11" s="8"/>
+        <v>15</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
UAT work 09/29/2023 -- UAT observations changes
</commit_message>
<xml_diff>
--- a/ui/src/assets/downloads/uat-scripts.xlsx
+++ b/ui/src/assets/downloads/uat-scripts.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Full time EE-Calendar view " sheetId="1" state="visible" r:id="rId2"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="44">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -89,6 +89,9 @@
   </si>
   <si>
     <t xml:space="preserve">As an Admin note down the working and non-working days of the associate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fail</t>
   </si>
   <si>
     <r>
@@ -529,7 +532,7 @@
         <v>15</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
@@ -543,10 +546,10 @@
         <v>4</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>15</v>
@@ -566,10 +569,10 @@
         <v>5</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>15</v>
@@ -589,10 +592,10 @@
         <v>6</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>15</v>
@@ -612,10 +615,10 @@
         <v>7</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>15</v>
@@ -635,10 +638,10 @@
         <v>8</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>15</v>
@@ -658,10 +661,10 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>15</v>
@@ -739,19 +742,19 @@
     </row>
     <row r="2" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>14</v>
@@ -800,13 +803,13 @@
         <v>20</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
@@ -820,10 +823,10 @@
         <v>4</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>15</v>
@@ -843,10 +846,10 @@
         <v>5</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>15</v>
@@ -866,10 +869,10 @@
         <v>6</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>15</v>
@@ -889,10 +892,10 @@
         <v>7</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>15</v>
@@ -912,10 +915,10 @@
         <v>8</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>15</v>
@@ -935,10 +938,10 @@
         <v>9</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>15</v>
@@ -958,10 +961,10 @@
         <v>10</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
UAT work 10/16/2023 -- UAT observations changes
</commit_message>
<xml_diff>
--- a/ui/src/assets/downloads/uat-scripts.xlsx
+++ b/ui/src/assets/downloads/uat-scripts.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Full time EE-Calendar view " sheetId="1" state="visible" r:id="rId2"/>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">The Associate's public profile will be displayed</t>
   </si>
   <si>
-    <t xml:space="preserve">As expected</t>
+    <t xml:space="preserve">As Expected</t>
   </si>
   <si>
     <t xml:space="preserve">Pass</t>
@@ -355,7 +355,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -390,6 +390,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -759,7 +763,7 @@
       <c r="F2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="9" t="s">
         <v>15</v>
       </c>
       <c r="H2" s="4" t="s">

</xml_diff>